<commit_message>
feat: update Product 24 Amazon redirect URL to B0HK7KMY51 and add detailed product listing content
</commit_message>
<xml_diff>
--- a/Guthani_Products_Catalog.xlsx
+++ b/Guthani_Products_Catalog.xlsx
@@ -1979,12 +1979,12 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Product 24</t>
+          <t>Guthni Handmade Round Woven Sling Bag with Pink Bow</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>A premium handcrafted piece from the Guthni Collection. Meticulously designed with traditional motifs and modern craftsmanship.</t>
+          <t>Add a touch of charm to your wardrobe with this beautiful handmade round woven handbag. Designed with a distinctive circular shape and an attractive pink bow, this bag combines traditional handcrafted appeal with a trendy contemporary look. The woven texture gives it a natural and elegant appearance, while the decorative bow adds a playful and stylish finish. Its convenient handle makes it comfortable to carry on your shoulder or by hand.</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
@@ -1994,37 +1994,37 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>Fine Handcrafted Jewellery</t>
+          <t>Natural-fiber woven material, fabric bow accent</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>Silver &amp; Gemstones</t>
+          <t>Natural fiber &amp; Pink bow</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>Standard / Adjustable</t>
+          <t>Standard Round Sling Bag</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>Hook-and-chain / Adjustable</t>
+          <t>Shoulder strap / Handheld</t>
         </is>
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>Pair with ethnic wear or contemporary outfits for an elegant style statement.</t>
+          <t>Style it with casual cotton dresses, kurtas, or everyday western outfits. Ideal for casual outings, parties, vacations, shopping, and daytime events.</t>
         </is>
       </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
-          <t>Store in an airtight zip-lock bag. Keep away from water, perfumes, and other chemicals.</t>
+          <t>Keep dry. Spot clean gently with a soft dry cloth. Avoid exposure to water, rain, and direct heat to protect the natural-fiber weave and fabric bow.</t>
         </is>
       </c>
       <c r="L25" s="2" t="inlineStr">
         <is>
-          <t>https://www.amazon.in</t>
+          <t>https://www.amazon.in/dp/B0HK7KMY51</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add products 31-36 and 38 with PDF spec metadata, update collection cards to show product names and View Now button, and remove on-image text overlays
</commit_message>
<xml_diff>
--- a/Guthani_Products_Catalog.xlsx
+++ b/Guthani_Products_Catalog.xlsx
@@ -452,7 +452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L29"/>
+  <dimension ref="A1:L39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -2269,6 +2269,606 @@
         </is>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>/new_webp_format_images/Product 29/H-007.jpg.jpeg</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>29</v>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Product 29</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>A premium handcrafted piece from the Guthni Collection. Meticulously designed with traditional motifs and modern craftsmanship.</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>Festive Edit, New Arrivals</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>Fine Handcrafted Jewellery</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>Silver &amp; Gemstones</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>Standard / Adjustable</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>Hook-and-chain / Adjustable</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>Pair with ethnic wear or contemporary outfits for an elegant style statement.</t>
+        </is>
+      </c>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>Store in an airtight zip-lock bag. Keep away from water, perfumes, and other chemicals.</t>
+        </is>
+      </c>
+      <c r="L30" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.in</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>/new_webp_format_images/Product 30/H-008.jpg.jpeg</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Product 30</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>A premium handcrafted piece from the Guthni Collection. Meticulously designed with traditional motifs and modern craftsmanship.</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>Festive Edit, New Arrivals</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>Fine Handcrafted Jewellery</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>Silver &amp; Gemstones</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>Standard / Adjustable</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>Hook-and-chain / Adjustable</t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>Pair with ethnic wear or contemporary outfits for an elegant style statement.</t>
+        </is>
+      </c>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>Store in an airtight zip-lock bag. Keep away from water, perfumes, and other chemicals.</t>
+        </is>
+      </c>
+      <c r="L31" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.in</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>/new_webp_format_images/Product 31/WhatsApp Image 2026-09-23 at 14.47.37.jpeg</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>31</v>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Guthni Handcrafted Royal Blue Crochet &amp; Cowrie Shell Choker</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Handcrafted ethnic bohemian choker necklace featuring an intricate royal blue fabric crochet center panel, tightly wrapped thread-coated light metal rod collar, genuine cowrie shells, traditional oxidized silver-toned cylindrical pendant, miniature bells, multi-colored seed bead strands, and dangling vintage-style coins.</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>Festive Edit, New Arrivals</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>Light metal rod coated with premium thread, handcrafted royal blue fabric crochet base, genuine cowrie shells, oxidized silver-toned cylindrical pendant, miniature bells, multi-colored seed beads, and vintage-style coin dangles</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>Royal Blue, Silver, and Multi-colored seed bead accents</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>15 to 16 inches (Adjustable collar fit)</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>Flexible open-ended choker collar</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>Perfectly complements ethnic wear, fusion outfits, sarees, kurtis, and bohemian-inspired casual clothing. Ideal for festive occasions, parties, and cultural events.</t>
+        </is>
+      </c>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>Store in a dry place away from moisture, perfumes, and direct chemicals. Wipe gently with a soft cotton cloth.</t>
+        </is>
+      </c>
+      <c r="L32" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.in</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>/new_webp_format_images/Product 32/WhatsApp Image 2026-09-23 at 15.13.26.jpeg</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>32</v>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>Guthni Handcrafted Gujarati Mirror Work &amp; Cowrie Shell Choker</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>Handcrafted traditional ethnic necklace featuring intricate thread embroidery, classic reflective mirror work, a rich fringe of natural cowrie shells (kaudi), and delicate pearl bead accents attached to a vibrant orange fabric-wrapped flexible neck wire.</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>Festive Edit, New Arrivals</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>Premium fabric, cotton thread, traditional mirrors, natural cowrie shells, and faux pearls</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>Vibrant Orange, Multicolor embroidery, and White pearls &amp; cowrie shells</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>15 to 16 inches (Choker / Short necklace fit)</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>Flexible neck wire collar style</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t>Perfect for traditional events, ethnic wear, Navratri, festive celebrations, cultural programs, parties, or bohemian-chic daily styling. Effortlessly complements sarees, lehengas, kurtis, and bohemian outfits.</t>
+        </is>
+      </c>
+      <c r="K33" s="2" t="inlineStr">
+        <is>
+          <t>Store in a dry place away from moisture, perfumes, and harsh chemicals. Handle mirror work and cowrie shells gently.</t>
+        </is>
+      </c>
+      <c r="L33" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.in</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>/new_webp_format_images/Product 33/WhatsApp Image 2026-09-23 at 15.25.01.jpeg</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>33</v>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Guthni Handcrafted Oxidized Silver Talisman Collar Necklace</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Authentic handcrafted ethnic statement collar necklace featuring a traditional oxidized silver-plated central amulet (tabiz) pendant, vintage-style coin charms, and dangling multi-strand multicolored bead fringes attached to a sturdy metal-core collar ring enclosed in soft thread wrapping.</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>Festive Edit, New Arrivals</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>Oxidized silver-plated metal core collar ring, alloy metal accents, and premium multi-colored glass seed beads</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>Oxidized Silver, Multicolored seed beads</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>15 to 16 inches (Adjustable open-collar fit)</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>Open-ended flexible collar ring with smooth metallic bead terminals</t>
+        </is>
+      </c>
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t>Perfect complement for traditional attire, festive wear, boho-chic outfits, and ethnic fusion styles.</t>
+        </is>
+      </c>
+      <c r="K34" s="2" t="inlineStr">
+        <is>
+          <t>Store in a dry place away from moisture, perfumes, and direct chemicals to maintain the oxidized silver finish.</t>
+        </is>
+      </c>
+      <c r="L34" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.in</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>/new_webp_format_images/Product 34/WhatsApp Image 2026-09-23 at 15.29.23.jpeg</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>34</v>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>Guthni Handcrafted Green Thread &amp; Cowrie Shell Statement Choker</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>Handcrafted statement choker necklace featuring a flexible green yarn-wrapped band adorned with an artistic floral cluster of genuine white cowrie shells, graceful silver-toned chains, smooth green resin beads, and a joyful cluster of multi-colored miniature ghungroos (bells) that create a soft chime.</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>Festive Edit, New Arrivals</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>Thread-wrapped metal ring, genuine cowrie shells, resin beads, metallic chains, and mini ghungroos (bells)</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>Green, White, and Multi-color Ghungroo accents</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>15 to 16 inches (Choker length)</t>
+        </is>
+      </c>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
+          <t>Slip-on / Flexible Band Style</t>
+        </is>
+      </c>
+      <c r="J35" s="2" t="inlineStr">
+        <is>
+          <t>Perfect accessory for traditional wear, Garba nights, ethnic festivals, cultural events, or casual fusion outfits.</t>
+        </is>
+      </c>
+      <c r="K35" s="2" t="inlineStr">
+        <is>
+          <t>Keep thread and cowrie shells dry. Store in a soft pouch away from moisture and perfumes.</t>
+        </is>
+      </c>
+      <c r="L35" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.in</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>/new_webp_format_images/Product 35/WhatsApp Image 2026-09-23 at 15.35.16.jpeg</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>35</v>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>Guthni Handcrafted Pink Thread Ring Necklace with Cowries &amp; Ghungroo</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>Expertly handcrafted ethnic statement necklace featuring a vibrant pink thread-wrapped flexible metal ring, complemented by multi-strand silver-toned chains adorned with natural cowrie shells, fabric thread balls, and traditional ghungroos.</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>Festive Edit, New Arrivals</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>Metal ring with premium pink thread wrapping, alloy chains, natural cowrie shells, thread balls, and metallic ghungroos (bells)</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>Vibrant Pink, Silver, and White cowrie shells</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>15 to 16 inches (Collar / Choker length)</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>Flexible Open-Ring Style</t>
+        </is>
+      </c>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t>Perfect accessory for ethnic wear, Navratri Garba outfits, bohemian fashion, cultural festivals, and casual styling.</t>
+        </is>
+      </c>
+      <c r="K36" s="2" t="inlineStr">
+        <is>
+          <t>Store in a dry place away from water and humidity. Clean gently with a soft dry cloth.</t>
+        </is>
+      </c>
+      <c r="L36" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.in</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>/new_webp_format_images/Product 36/WhatsApp Image 2026-09-23 at 15.38.35.jpeg</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>36</v>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>Guthni Handcrafted Yellow Textile &amp; Faux Pearl Collar Necklace with Gold Coins</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>Handcrafted statement necklace featuring a sturdy metal ring meticulously wrapped in bright yellow textile yarn, finished with sleek silver-tone metallic bead ends. The centerpiece showcases an artistic cluster of lustrous faux pearls bordered by intricate, antique-finish gold coins.</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>Festive Edit, New Arrivals</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>Metal core ring, high-quality yellow textile yarn, artificial pearls, and antique-finish metallic coins</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>Bright Yellow, Gold, and White Pearls</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>15 to 16 inches (Collar length)</t>
+        </is>
+      </c>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t>Open-end flexible collar style with metallic bead finials</t>
+        </is>
+      </c>
+      <c r="J37" s="2" t="inlineStr">
+        <is>
+          <t>An ideal accessory for festive celebrations, traditional functions, ethnic gatherings, kurtis, sarees, or fusion wear.</t>
+        </is>
+      </c>
+      <c r="K37" s="2" t="inlineStr">
+        <is>
+          <t>Keep away from water and harsh chemicals. Store flat in a dry box or soft pouch.</t>
+        </is>
+      </c>
+      <c r="L37" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.in</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>/new_webp_format_images/Product 37/WhatsApp Image 2026-09-21 at 15.33.07.jpeg</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>37</v>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>Product 37</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>A premium handcrafted piece from the Guthni Collection. Meticulously designed with traditional motifs and modern craftsmanship.</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>Festive Edit, New Arrivals</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>Fine Handcrafted Jewellery</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>Silver &amp; Gemstones</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>Standard / Adjustable</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>Hook-and-chain / Adjustable</t>
+        </is>
+      </c>
+      <c r="J38" s="2" t="inlineStr">
+        <is>
+          <t>Pair with ethnic wear or contemporary outfits for an elegant style statement.</t>
+        </is>
+      </c>
+      <c r="K38" s="2" t="inlineStr">
+        <is>
+          <t>Store in an airtight zip-lock bag. Keep away from water, perfumes, and other chemicals.</t>
+        </is>
+      </c>
+      <c r="L38" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.in</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>/new_webp_format_images/Product 38/WhatsApp Image 2026-09-23 at 14.46.38.jpeg</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>38</v>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>Guthni Handcrafted Multicolour Beaded Statement Necklace</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>Handmade statement necklace featuring a bright yellow lightweight metal neckpiece decorated with multiple strands of colourful beads and assorted hanging decorative pendants and charms, creating a playful, bohemian and eye-catching look.</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>Festive Edit, New Arrivals</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>Yellow lightweight metal neckpiece, multicolour decorative beads, and assorted hanging charms &amp; pendants</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>Yellow neckpiece, Multicolour beads &amp; charms</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>15 to 16 inches</t>
+        </is>
+      </c>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t>Slip-on / Open-collar style</t>
+        </is>
+      </c>
+      <c r="J39" s="2" t="inlineStr">
+        <is>
+          <t>Suitable for casual outings, festive occasions, parties, traditional Indian outfits, fusion wear, kurtis, dresses or casual clothing.</t>
+        </is>
+      </c>
+      <c r="K39" s="2" t="inlineStr">
+        <is>
+          <t>Store in a dry place. Clean gently with a soft cloth. Keep away from water and perfumes.</t>
+        </is>
+      </c>
+      <c r="L39" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.in</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: add Amazon product redirect links for products 31, 32, 33, 34, 35, and 38
</commit_message>
<xml_diff>
--- a/Guthani_Products_Catalog.xlsx
+++ b/Guthani_Products_Catalog.xlsx
@@ -2445,7 +2445,7 @@
       </c>
       <c r="L32" s="2" t="inlineStr">
         <is>
-          <t>https://www.amazon.in</t>
+          <t>https://www.amazon.in/dp/B0HL363426</t>
         </is>
       </c>
     </row>
@@ -2505,7 +2505,7 @@
       </c>
       <c r="L33" s="2" t="inlineStr">
         <is>
-          <t>https://www.amazon.in</t>
+          <t>https://www.amazon.in/dp/B0HL3C413F</t>
         </is>
       </c>
     </row>
@@ -2565,7 +2565,7 @@
       </c>
       <c r="L34" s="2" t="inlineStr">
         <is>
-          <t>https://www.amazon.in</t>
+          <t>https://www.amazon.in/dp/B0HL464QK8</t>
         </is>
       </c>
     </row>
@@ -2625,7 +2625,7 @@
       </c>
       <c r="L35" s="2" t="inlineStr">
         <is>
-          <t>https://www.amazon.in</t>
+          <t>https://www.amazon.in/dp/B0HL3CHZYK</t>
         </is>
       </c>
     </row>
@@ -2685,7 +2685,7 @@
       </c>
       <c r="L36" s="2" t="inlineStr">
         <is>
-          <t>https://www.amazon.in</t>
+          <t>https://www.amazon.in/dp/B0HL3BTQGW</t>
         </is>
       </c>
     </row>
@@ -2865,7 +2865,7 @@
       </c>
       <c r="L39" s="2" t="inlineStr">
         <is>
-          <t>https://www.amazon.in</t>
+          <t>https://www.amazon.in/dp/B0HL3LLWQD</t>
         </is>
       </c>
     </row>

</xml_diff>